<commit_message>
Fixed latitude and longitude in sinks sheet
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -1,30 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shamm\OneDrive\Desktop\ExxonSupplyChainRice2026\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28DF7180-329D-4053-83CC-839B8A7B2356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sources" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Sinks" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Edges" sheetId="3" r:id="rId7"/>
+    <sheet name="Sources" sheetId="1" r:id="rId1"/>
+    <sheet name="Sinks" sheetId="2" r:id="rId2"/>
+    <sheet name="Edges" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={9657acb3-d37a-49c5-ada1-034a7516d7cb}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{9657acb3-d37a-49c5-ada1-034a7516d7cb}" ref="M1">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{9657ACB3-D37A-49C5-ADA1-034A7516D7CB}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-	50% liquid caustic has density of ~1.52g/cm3
-</t>
+    50% liquid caustic has density of ~1.52g/cm3</t>
       </text>
     </comment>
   </commentList>
@@ -235,40 +256,42 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color theme="0"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <i/>
-      <sz val="9.0"/>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -279,7 +302,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -289,11 +312,21 @@
     </fill>
   </fills>
   <borders count="3">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -302,87 +335,78 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="16">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" vertical="bottom"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
-<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Shammas Ahmed" id="{7149d9b8-27be-4ac8-8663-693842e25966}" providerId="google-sheets"/>
-</x18tc:personList>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Shammas Ahmed" id="{7149D9B8-27BE-4AC8-8663-693842E25966}" userId="" providerId="google-sheets"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -572,34 +596,37 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="M1" dT="2026-10-03T21:19:56.00" personId="{7149d9b8-27be-4ac8-8663-693842e25966}" id="{9657acb3-d37a-49c5-ada1-034a7516d7cb}" done="0">
-    <x18tc:text xml:space="preserve">50% liquid caustic has density of ~1.52g/cm3</x18tc:text>
-  </x18tc:threadedComment>
-</x18tc:ThreadedComments>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="M1" dT="2026-10-03T21:19:56.00" personId="{7149D9B8-27BE-4AC8-8663-693842E25966}" id="{9657ACB3-D37A-49C5-ADA1-034A7516D7CB}">
+    <text>50% liquid caustic has density of ~1.52g/cm3</text>
+  </threadedComment>
+</ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Y11"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="32.5"/>
-    <col customWidth="1" min="7" max="7" width="24.75"/>
-    <col customWidth="1" min="8" max="8" width="23.13"/>
-    <col customWidth="1" min="9" max="9" width="15.88"/>
-    <col customWidth="1" min="10" max="10" width="16.5"/>
-    <col customWidth="1" min="11" max="11" width="16.88"/>
-    <col customWidth="1" min="12" max="12" width="15.88"/>
+    <col min="1" max="1" width="32.44140625" customWidth="1"/>
+    <col min="7" max="7" width="24.77734375" customWidth="1"/>
+    <col min="8" max="8" width="23.109375" customWidth="1"/>
+    <col min="9" max="9" width="15.88671875" customWidth="1"/>
+    <col min="10" max="10" width="16.44140625" customWidth="1"/>
+    <col min="11" max="11" width="16.88671875" customWidth="1"/>
+    <col min="12" max="12" width="15.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -650,7 +677,7 @@
       <c r="X1" s="3"/>
       <c r="Y1" s="3"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
@@ -664,34 +691,34 @@
         <v>15</v>
       </c>
       <c r="E2" s="5">
-        <v>-95.3597</v>
+        <v>-95.359700000000004</v>
       </c>
       <c r="F2" s="5">
         <v>28.9543</v>
       </c>
       <c r="G2" s="6">
-        <v>2250000.0</v>
+        <v>2250000</v>
       </c>
       <c r="H2" s="6">
-        <v>2640000.0</v>
+        <v>2640000</v>
       </c>
       <c r="I2" s="6">
-        <v>2940000.0</v>
+        <v>2940000</v>
       </c>
       <c r="J2" s="7">
-        <f t="shared" ref="J2:L2" si="1">G2*1.10231</f>
+        <f t="shared" ref="J2:L2" si="0">G2*1.10231</f>
         <v>2480197.5</v>
       </c>
       <c r="K2" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2910098.4</v>
       </c>
       <c r="L2" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3240791.4</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
@@ -705,34 +732,34 @@
         <v>15</v>
       </c>
       <c r="E3" s="5">
-        <v>-93.2842</v>
+        <v>-93.284199999999998</v>
       </c>
       <c r="F3" s="5">
-        <v>30.2131</v>
+        <v>30.213100000000001</v>
       </c>
       <c r="G3" s="6">
-        <v>900000.0</v>
+        <v>900000</v>
       </c>
       <c r="H3" s="6">
-        <v>1056000.0</v>
+        <v>1056000</v>
       </c>
       <c r="I3" s="6">
-        <v>1176000.0</v>
+        <v>1176000</v>
       </c>
       <c r="J3" s="7">
-        <f t="shared" ref="J3:L3" si="2">G3*1.10231</f>
-        <v>992079</v>
+        <f t="shared" ref="J3:L3" si="1">G3*1.10231</f>
+        <v>992078.99999999988</v>
       </c>
       <c r="K3" s="7">
-        <f t="shared" si="2"/>
-        <v>1164039.36</v>
+        <f t="shared" si="1"/>
+        <v>1164039.3599999999</v>
       </c>
       <c r="L3" s="7">
-        <f t="shared" si="2"/>
-        <v>1296316.56</v>
-      </c>
-    </row>
-    <row r="4">
+        <f t="shared" si="1"/>
+        <v>1296316.5599999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>19</v>
       </c>
@@ -746,34 +773,34 @@
         <v>15</v>
       </c>
       <c r="E4" s="5">
-        <v>-91.223</v>
+        <v>-91.222999999999999</v>
       </c>
       <c r="F4" s="5">
-        <v>30.268</v>
+        <v>30.268000000000001</v>
       </c>
       <c r="G4" s="6">
-        <v>750000.0</v>
+        <v>750000</v>
       </c>
       <c r="H4" s="6">
-        <v>880000.0</v>
+        <v>880000</v>
       </c>
       <c r="I4" s="6">
-        <v>980000.0</v>
+        <v>980000</v>
       </c>
       <c r="J4" s="7">
-        <f t="shared" ref="J4:L4" si="3">G4*1.10231</f>
-        <v>826732.5</v>
+        <f t="shared" ref="J4:L4" si="2">G4*1.10231</f>
+        <v>826732.49999999988</v>
       </c>
       <c r="K4" s="7">
-        <f t="shared" si="3"/>
-        <v>970032.8</v>
+        <f t="shared" si="2"/>
+        <v>970032.79999999993</v>
       </c>
       <c r="L4" s="7">
-        <f t="shared" si="3"/>
-        <v>1080263.8</v>
-      </c>
-    </row>
-    <row r="5">
+        <f t="shared" si="2"/>
+        <v>1080263.7999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>21</v>
       </c>
@@ -787,34 +814,34 @@
         <v>15</v>
       </c>
       <c r="E5" s="5">
-        <v>-91.2215</v>
+        <v>-91.221500000000006</v>
       </c>
       <c r="F5" s="5">
-        <v>30.2522</v>
+        <v>30.252199999999998</v>
       </c>
       <c r="G5" s="6">
-        <v>637500.0</v>
+        <v>637500</v>
       </c>
       <c r="H5" s="6">
-        <v>748000.0</v>
+        <v>748000</v>
       </c>
       <c r="I5" s="6">
-        <v>833000.0</v>
+        <v>833000</v>
       </c>
       <c r="J5" s="7">
-        <f t="shared" ref="J5:L5" si="4">G5*1.10231</f>
-        <v>702722.625</v>
+        <f t="shared" ref="J5:L5" si="3">G5*1.10231</f>
+        <v>702722.62499999988</v>
       </c>
       <c r="K5" s="7">
-        <f t="shared" si="4"/>
-        <v>824527.88</v>
+        <f t="shared" si="3"/>
+        <v>824527.87999999989</v>
       </c>
       <c r="L5" s="7">
-        <f t="shared" si="4"/>
-        <v>918224.23</v>
-      </c>
-    </row>
-    <row r="6">
+        <f t="shared" si="3"/>
+        <v>918224.22999999986</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>22</v>
       </c>
@@ -828,34 +855,34 @@
         <v>15</v>
       </c>
       <c r="E6" s="5">
-        <v>-96.5583</v>
+        <v>-96.558300000000003</v>
       </c>
       <c r="F6" s="5">
-        <v>28.6942</v>
+        <v>28.694199999999999</v>
       </c>
       <c r="G6" s="6">
-        <v>600000.0</v>
+        <v>600000</v>
       </c>
       <c r="H6" s="6">
-        <v>704000.0</v>
+        <v>704000</v>
       </c>
       <c r="I6" s="6">
-        <v>784000.0</v>
+        <v>784000</v>
       </c>
       <c r="J6" s="7">
-        <f t="shared" ref="J6:L6" si="5">G6*1.10231</f>
-        <v>661386</v>
+        <f t="shared" ref="J6:L6" si="4">G6*1.10231</f>
+        <v>661385.99999999988</v>
       </c>
       <c r="K6" s="7">
-        <f t="shared" si="5"/>
-        <v>776026.24</v>
+        <f t="shared" si="4"/>
+        <v>776026.23999999987</v>
       </c>
       <c r="L6" s="7">
-        <f t="shared" si="5"/>
-        <v>864211.04</v>
-      </c>
-    </row>
-    <row r="7">
+        <f t="shared" si="4"/>
+        <v>864211.03999999992</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>24</v>
       </c>
@@ -869,34 +896,34 @@
         <v>15</v>
       </c>
       <c r="E7" s="5">
-        <v>-90.4578</v>
+        <v>-90.457800000000006</v>
       </c>
       <c r="F7" s="5">
-        <v>29.9928</v>
+        <v>29.992799999999999</v>
       </c>
       <c r="G7" s="6">
-        <v>562500.0</v>
+        <v>562500</v>
       </c>
       <c r="H7" s="6">
-        <v>660000.0</v>
+        <v>660000</v>
       </c>
       <c r="I7" s="6">
-        <v>735000.0</v>
+        <v>735000</v>
       </c>
       <c r="J7" s="7">
-        <f t="shared" ref="J7:L7" si="6">G7*1.10231</f>
+        <f t="shared" ref="J7:L7" si="5">G7*1.10231</f>
         <v>620049.375</v>
       </c>
       <c r="K7" s="7">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>727524.6</v>
       </c>
       <c r="L7" s="7">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>810197.85</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>26</v>
       </c>
@@ -913,31 +940,31 @@
         <v>-91.0261</v>
       </c>
       <c r="F8" s="5">
-        <v>30.2223</v>
+        <v>30.222300000000001</v>
       </c>
       <c r="G8" s="6">
-        <v>525000.0</v>
+        <v>525000</v>
       </c>
       <c r="H8" s="6">
-        <v>616000.0</v>
+        <v>616000</v>
       </c>
       <c r="I8" s="6">
-        <v>686000.0</v>
+        <v>686000</v>
       </c>
       <c r="J8" s="7">
-        <f t="shared" ref="J8:L8" si="7">G8*1.10231</f>
+        <f t="shared" ref="J8:L8" si="6">G8*1.10231</f>
         <v>578712.75</v>
       </c>
       <c r="K8" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>679022.96</v>
       </c>
       <c r="L8" s="7">
-        <f t="shared" si="7"/>
-        <v>756184.66</v>
-      </c>
-    </row>
-    <row r="9">
+        <f t="shared" si="6"/>
+        <v>756184.65999999992</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>28</v>
       </c>
@@ -951,34 +978,34 @@
         <v>15</v>
       </c>
       <c r="E9" s="5">
-        <v>-88.0336</v>
+        <v>-88.033600000000007</v>
       </c>
       <c r="F9" s="5">
-        <v>31.2688</v>
+        <v>31.268799999999999</v>
       </c>
       <c r="G9" s="6">
-        <v>450000.0</v>
+        <v>450000</v>
       </c>
       <c r="H9" s="6">
-        <v>528000.0</v>
+        <v>528000</v>
       </c>
       <c r="I9" s="6">
-        <v>588000.0</v>
+        <v>588000</v>
       </c>
       <c r="J9" s="7">
-        <f t="shared" ref="J9:L9" si="8">G9*1.10231</f>
-        <v>496039.5</v>
+        <f t="shared" ref="J9:L9" si="7">G9*1.10231</f>
+        <v>496039.49999999994</v>
       </c>
       <c r="K9" s="7">
-        <f t="shared" si="8"/>
-        <v>582019.68</v>
+        <f t="shared" si="7"/>
+        <v>582019.67999999993</v>
       </c>
       <c r="L9" s="7">
-        <f t="shared" si="8"/>
-        <v>648158.28</v>
-      </c>
-    </row>
-    <row r="10">
+        <f t="shared" si="7"/>
+        <v>648158.27999999991</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>31</v>
       </c>
@@ -992,34 +1019,34 @@
         <v>15</v>
       </c>
       <c r="E10" s="5">
-        <v>-97.2289</v>
+        <v>-97.228899999999996</v>
       </c>
       <c r="F10" s="5">
         <v>27.8828</v>
       </c>
       <c r="G10" s="6">
-        <v>412500.0</v>
+        <v>412500</v>
       </c>
       <c r="H10" s="6">
-        <v>484000.0</v>
+        <v>484000</v>
       </c>
       <c r="I10" s="6">
-        <v>539000.0</v>
+        <v>539000</v>
       </c>
       <c r="J10" s="7">
-        <f t="shared" ref="J10:L10" si="9">G10*1.10231</f>
-        <v>454702.875</v>
+        <f t="shared" ref="J10:L10" si="8">G10*1.10231</f>
+        <v>454702.87499999994</v>
       </c>
       <c r="K10" s="7">
-        <f t="shared" si="9"/>
-        <v>533518.04</v>
+        <f t="shared" si="8"/>
+        <v>533518.03999999992</v>
       </c>
       <c r="L10" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>594145.09</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
@@ -1033,57 +1060,58 @@
         <v>15</v>
       </c>
       <c r="E11" s="5">
-        <v>-88.3512</v>
+        <v>-88.351200000000006</v>
       </c>
       <c r="F11" s="5">
-        <v>37.0345</v>
+        <v>37.034500000000001</v>
       </c>
       <c r="G11" s="6">
-        <v>337500.0</v>
+        <v>337500</v>
       </c>
       <c r="H11" s="6">
-        <v>396000.0</v>
+        <v>396000</v>
       </c>
       <c r="I11" s="6">
-        <v>441000.0</v>
+        <v>441000</v>
       </c>
       <c r="J11" s="7">
-        <f t="shared" ref="J11:L11" si="10">G11*1.10231</f>
-        <v>372029.625</v>
+        <f t="shared" ref="J11:L11" si="9">G11*1.10231</f>
+        <v>372029.62499999994</v>
       </c>
       <c r="K11" s="7">
-        <f t="shared" si="10"/>
-        <v>436514.76</v>
+        <f t="shared" si="9"/>
+        <v>436514.75999999995</v>
       </c>
       <c r="L11" s="7">
-        <f t="shared" si="10"/>
-        <v>486118.71</v>
+        <f t="shared" si="9"/>
+        <v>486118.70999999996</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:AB21"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="30.75"/>
-    <col customWidth="1" min="2" max="2" width="29.63"/>
-    <col customWidth="1" min="3" max="3" width="10.25"/>
-    <col customWidth="1" min="5" max="5" width="11.5"/>
-    <col customWidth="1" min="6" max="6" width="10.63"/>
-    <col customWidth="1" min="7" max="7" width="19.13"/>
-    <col customWidth="1" min="8" max="8" width="19.88"/>
-    <col customWidth="1" min="9" max="9" width="21.13"/>
-    <col customWidth="1" min="10" max="13" width="19.13"/>
+    <col min="1" max="1" width="30.77734375" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="3" max="3" width="10.21875" customWidth="1"/>
+    <col min="5" max="5" width="11.44140625" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19.109375" customWidth="1"/>
+    <col min="8" max="8" width="19.88671875" customWidth="1"/>
+    <col min="9" max="9" width="21.109375" customWidth="1"/>
+    <col min="10" max="13" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -1139,7 +1167,7 @@
       <c r="AA1" s="3"/>
       <c r="AB1" s="3"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>44</v>
       </c>
@@ -1152,39 +1180,39 @@
       <c r="D2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="8">
-        <v>70.2552</v>
-      </c>
-      <c r="F2" s="8">
-        <v>-148.3384</v>
+      <c r="E2" s="15">
+        <v>-148.33840000000001</v>
+      </c>
+      <c r="F2" s="15">
+        <v>70.255200000000002</v>
       </c>
       <c r="G2" s="9">
-        <v>600.0</v>
+        <v>600</v>
       </c>
       <c r="H2" s="10">
-        <v>1200.0</v>
+        <v>1200</v>
       </c>
       <c r="I2" s="10">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="J2" s="11">
-        <f t="shared" ref="J2:L2" si="1">G2*1.10231</f>
-        <v>661.386</v>
+        <f t="shared" ref="J2:L2" si="0">G2*1.10231</f>
+        <v>661.38599999999997</v>
       </c>
       <c r="K2" s="10">
-        <f t="shared" si="1"/>
-        <v>1322.772</v>
+        <f t="shared" si="0"/>
+        <v>1322.7719999999999</v>
       </c>
       <c r="L2" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2204.62</v>
       </c>
       <c r="M2" s="12">
-        <v>380000.0</v>
+        <v>380000</v>
       </c>
       <c r="N2" s="13"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>47</v>
       </c>
@@ -1197,39 +1225,39 @@
       <c r="D3" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="8">
-        <v>30.6033</v>
-      </c>
-      <c r="F3" s="8">
-        <v>-87.2711</v>
+      <c r="E3" s="15">
+        <v>-87.271100000000004</v>
+      </c>
+      <c r="F3" s="15">
+        <v>30.603300000000001</v>
       </c>
       <c r="G3" s="9">
-        <v>400.0</v>
+        <v>400</v>
       </c>
       <c r="H3" s="8">
-        <v>800.0</v>
+        <v>800</v>
       </c>
       <c r="I3" s="10">
-        <v>1300.0</v>
+        <v>1300</v>
       </c>
       <c r="J3" s="11">
-        <f t="shared" ref="J3:L3" si="2">G3*1.10231</f>
-        <v>440.924</v>
+        <f t="shared" ref="J3:L3" si="1">G3*1.10231</f>
+        <v>440.92399999999998</v>
       </c>
       <c r="K3" s="10">
-        <f t="shared" si="2"/>
-        <v>881.848</v>
+        <f t="shared" si="1"/>
+        <v>881.84799999999996</v>
       </c>
       <c r="L3" s="10">
-        <f t="shared" si="2"/>
-        <v>1433.003</v>
+        <f t="shared" si="1"/>
+        <v>1433.0029999999999</v>
       </c>
       <c r="M3" s="12">
-        <v>250000.0</v>
+        <v>250000</v>
       </c>
       <c r="N3" s="13"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>50</v>
       </c>
@@ -1242,39 +1270,39 @@
       <c r="D4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="8">
-        <v>41.4286</v>
-      </c>
-      <c r="F4" s="8">
-        <v>-88.1803</v>
+      <c r="E4" s="15">
+        <v>-88.180300000000003</v>
+      </c>
+      <c r="F4" s="15">
+        <v>41.428600000000003</v>
       </c>
       <c r="G4" s="11">
-        <v>3500.0</v>
+        <v>3500</v>
       </c>
       <c r="H4" s="10">
-        <v>5500.0</v>
+        <v>5500</v>
       </c>
       <c r="I4" s="10">
-        <v>8000.0</v>
+        <v>8000</v>
       </c>
       <c r="J4" s="11">
-        <f t="shared" ref="J4:L4" si="3">G4*1.10231</f>
-        <v>3858.085</v>
+        <f t="shared" ref="J4:L4" si="2">G4*1.10231</f>
+        <v>3858.0849999999996</v>
       </c>
       <c r="K4" s="10">
-        <f t="shared" si="3"/>
-        <v>6062.705</v>
+        <f t="shared" si="2"/>
+        <v>6062.704999999999</v>
       </c>
       <c r="L4" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>8818.48</v>
       </c>
       <c r="M4" s="12">
-        <v>1730000.0</v>
+        <v>1730000</v>
       </c>
       <c r="N4" s="13"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>53</v>
       </c>
@@ -1287,39 +1315,39 @@
       <c r="D5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="8">
-        <v>30.4851</v>
-      </c>
-      <c r="F5" s="8">
-        <v>-91.1895</v>
+      <c r="E5" s="15">
+        <v>-91.189499999999995</v>
+      </c>
+      <c r="F5" s="15">
+        <v>30.485099999999999</v>
       </c>
       <c r="G5" s="11">
-        <v>10000.0</v>
+        <v>10000</v>
       </c>
       <c r="H5" s="10">
-        <v>15000.0</v>
+        <v>15000</v>
       </c>
       <c r="I5" s="10">
-        <v>21000.0</v>
+        <v>21000</v>
       </c>
       <c r="J5" s="11">
-        <f t="shared" ref="J5:L5" si="4">G5*1.10231</f>
-        <v>11023.1</v>
+        <f t="shared" ref="J5:L5" si="3">G5*1.10231</f>
+        <v>11023.099999999999</v>
       </c>
       <c r="K5" s="10">
-        <f t="shared" si="4"/>
-        <v>16534.65</v>
+        <f t="shared" si="3"/>
+        <v>16534.649999999998</v>
       </c>
       <c r="L5" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>23148.51</v>
       </c>
       <c r="M5" s="12">
-        <v>4710000.0</v>
+        <v>4710000</v>
       </c>
       <c r="N5" s="13"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>55</v>
       </c>
@@ -1332,39 +1360,39 @@
       <c r="D6" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="15">
+        <v>-74.225099999999998</v>
+      </c>
+      <c r="F6" s="15">
         <v>40.6387</v>
       </c>
-      <c r="F6" s="8">
-        <v>-74.2251</v>
-      </c>
       <c r="G6" s="9">
-        <v>800.0</v>
+        <v>800</v>
       </c>
       <c r="H6" s="10">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="I6" s="10">
-        <v>2500.0</v>
+        <v>2500</v>
       </c>
       <c r="J6" s="11">
-        <f t="shared" ref="J6:L6" si="5">G6*1.10231</f>
-        <v>881.848</v>
+        <f t="shared" ref="J6:L6" si="4">G6*1.10231</f>
+        <v>881.84799999999996</v>
       </c>
       <c r="K6" s="10">
-        <f t="shared" si="5"/>
-        <v>1653.465</v>
+        <f t="shared" si="4"/>
+        <v>1653.4649999999999</v>
       </c>
       <c r="L6" s="10">
-        <f t="shared" si="5"/>
-        <v>2755.775</v>
+        <f t="shared" si="4"/>
+        <v>2755.7749999999996</v>
       </c>
       <c r="M6" s="12">
-        <v>470000.0</v>
+        <v>470000</v>
       </c>
       <c r="N6" s="13"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>58</v>
       </c>
@@ -1377,39 +1405,39 @@
       <c r="D7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="8">
-        <v>29.7402</v>
-      </c>
-      <c r="F7" s="8">
-        <v>-95.0118</v>
+      <c r="E7" s="15">
+        <v>-95.011799999999994</v>
+      </c>
+      <c r="F7" s="15">
+        <v>29.740200000000002</v>
       </c>
       <c r="G7" s="11">
-        <v>12000.0</v>
+        <v>12000</v>
       </c>
       <c r="H7" s="10">
-        <v>18000.0</v>
+        <v>18000</v>
       </c>
       <c r="I7" s="10">
-        <v>25000.0</v>
+        <v>25000</v>
       </c>
       <c r="J7" s="11">
-        <f t="shared" ref="J7:L7" si="6">G7*1.10231</f>
+        <f t="shared" ref="J7:L7" si="5">G7*1.10231</f>
         <v>13227.72</v>
       </c>
       <c r="K7" s="10">
-        <f t="shared" si="6"/>
-        <v>19841.58</v>
+        <f t="shared" si="5"/>
+        <v>19841.579999999998</v>
       </c>
       <c r="L7" s="10">
-        <f t="shared" si="6"/>
-        <v>27557.75</v>
+        <f t="shared" si="5"/>
+        <v>27557.749999999996</v>
       </c>
       <c r="M7" s="12">
-        <v>5650000.0</v>
+        <v>5650000</v>
       </c>
       <c r="N7" s="13"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>60</v>
       </c>
@@ -1422,39 +1450,39 @@
       <c r="D8" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="8">
-        <v>30.0683</v>
-      </c>
-      <c r="F8" s="8">
-        <v>-94.0847</v>
+      <c r="E8" s="15">
+        <v>-94.084699999999998</v>
+      </c>
+      <c r="F8" s="15">
+        <v>30.068300000000001</v>
       </c>
       <c r="G8" s="11">
-        <v>11000.0</v>
+        <v>11000</v>
       </c>
       <c r="H8" s="10">
-        <v>16500.0</v>
+        <v>16500</v>
       </c>
       <c r="I8" s="10">
-        <v>23000.0</v>
+        <v>23000</v>
       </c>
       <c r="J8" s="11">
-        <f t="shared" ref="J8:L8" si="7">G8*1.10231</f>
-        <v>12125.41</v>
+        <f t="shared" ref="J8:L8" si="6">G8*1.10231</f>
+        <v>12125.409999999998</v>
       </c>
       <c r="K8" s="10">
-        <f t="shared" si="7"/>
-        <v>18188.115</v>
+        <f t="shared" si="6"/>
+        <v>18188.114999999998</v>
       </c>
       <c r="L8" s="10">
-        <f t="shared" si="7"/>
-        <v>25353.13</v>
+        <f t="shared" si="6"/>
+        <v>25353.129999999997</v>
       </c>
       <c r="M8" s="12">
-        <v>5180000.0</v>
+        <v>5180000</v>
       </c>
       <c r="N8" s="13"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>62</v>
       </c>
@@ -1467,39 +1495,39 @@
       <c r="D9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="8">
-        <v>29.8378</v>
-      </c>
-      <c r="F9" s="8">
-        <v>-94.8872</v>
+      <c r="E9" s="15">
+        <v>-94.887200000000007</v>
+      </c>
+      <c r="F9" s="15">
+        <v>29.837800000000001</v>
       </c>
       <c r="G9" s="9">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="H9" s="10">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
       <c r="I9" s="10">
-        <v>1800.0</v>
+        <v>1800</v>
       </c>
       <c r="J9" s="11">
-        <f t="shared" ref="J9:L9" si="8">G9*1.10231</f>
-        <v>551.155</v>
+        <f t="shared" ref="J9:L9" si="7">G9*1.10231</f>
+        <v>551.15499999999997</v>
       </c>
       <c r="K9" s="10">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>1102.31</v>
       </c>
       <c r="L9" s="10">
-        <f t="shared" si="8"/>
-        <v>1984.158</v>
+        <f t="shared" si="7"/>
+        <v>1984.1579999999999</v>
       </c>
       <c r="M9" s="12">
-        <v>310000.0</v>
+        <v>310000</v>
       </c>
       <c r="N9" s="13"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>64</v>
       </c>
@@ -1512,54 +1540,91 @@
       <c r="D10" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="8">
-        <v>27.915</v>
-      </c>
-      <c r="F10" s="8">
-        <v>-97.2883</v>
+      <c r="E10" s="15">
+        <v>-97.288300000000007</v>
+      </c>
+      <c r="F10" s="15">
+        <v>27.914999999999999</v>
       </c>
       <c r="G10" s="11">
-        <v>2500.0</v>
+        <v>2500</v>
       </c>
       <c r="H10" s="10">
-        <v>4000.0</v>
+        <v>4000</v>
       </c>
       <c r="I10" s="10">
-        <v>6000.0</v>
+        <v>6000</v>
       </c>
       <c r="J10" s="11">
-        <f t="shared" ref="J10:L10" si="9">G10*1.10231</f>
-        <v>2755.775</v>
+        <f t="shared" ref="J10:L10" si="8">G10*1.10231</f>
+        <v>2755.7749999999996</v>
       </c>
       <c r="K10" s="10">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>4409.24</v>
       </c>
       <c r="L10" s="10">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>6613.86</v>
       </c>
       <c r="M10" s="12">
-        <v>1250000.0</v>
+        <v>1250000</v>
       </c>
       <c r="N10" s="13"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="E12" s="8"/>
       <c r="M12" s="14"/>
     </row>
+    <row r="13" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+    </row>
+    <row r="14" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+    </row>
+    <row r="15" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+    </row>
+    <row r="16" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+    </row>
+    <row r="17" spans="5:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+    </row>
+    <row r="18" spans="5:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+    </row>
+    <row r="19" spans="5:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+    </row>
+    <row r="20" spans="5:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+    </row>
+    <row r="21" spans="5:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="8"/>
+    </row>
   </sheetData>
-  <drawing r:id="rId4"/>
-  <legacyDrawing r:id="rId5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated canada lat long vals
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/166e7fef95bdf10f/Desktop/ExxonSupplyChainRice2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vivia/RICE/Fall 2026/CMOR 492/ExxonSupplyChainRice2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{28DF7180-329D-4053-83CC-839B8A7B2356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AADB314-361B-4550-BA22-3881499CA6CA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4557C59-DDEE-E246-8157-4B7AB989130F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="23560" windowHeight="12420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="1" r:id="rId1"/>
     <sheet name="Sinks" sheetId="2" r:id="rId2"/>
     <sheet name="Edges" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -26,7 +26,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="52">
   <si>
     <t>Name</t>
   </si>
@@ -158,13 +157,46 @@
   </si>
   <si>
     <t>Lemont</t>
+  </si>
+  <si>
+    <t>Strathcona Refinery</t>
+  </si>
+  <si>
+    <t>Edmonton</t>
+  </si>
+  <si>
+    <t>Alberta</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>Nanticoke Refinery</t>
+  </si>
+  <si>
+    <t>Nanticoke</t>
+  </si>
+  <si>
+    <t>Ontario</t>
+  </si>
+  <si>
+    <t>Sarnia Refinery</t>
+  </si>
+  <si>
+    <t>Sarnia</t>
+  </si>
+  <si>
+    <t>Cold Lake</t>
+  </si>
+  <si>
+    <t>Kearl</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -176,6 +208,7 @@
       <sz val="12"/>
       <color theme="0"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -183,18 +216,28 @@
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF616161"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -232,7 +275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -262,6 +305,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,18 +529,18 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Y6"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="32.44140625" customWidth="1"/>
-    <col min="7" max="7" width="24.77734375" customWidth="1"/>
-    <col min="8" max="8" width="23.109375" customWidth="1"/>
-    <col min="9" max="9" width="15.88671875" customWidth="1"/>
-    <col min="10" max="10" width="16.44140625" customWidth="1"/>
-    <col min="11" max="11" width="16.88671875" customWidth="1"/>
-    <col min="12" max="12" width="15.88671875" customWidth="1"/>
+    <col min="1" max="1" width="32.5" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="23.1640625" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.5" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" ht="51" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -547,7 +591,7 @@
       <c r="X1" s="3"/>
       <c r="Y1" s="3"/>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="13" x14ac:dyDescent="0.15">
       <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
@@ -591,7 +635,7 @@
         <v>6722.2469178361807</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="13" x14ac:dyDescent="0.15">
       <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
@@ -635,7 +679,7 @@
         <v>5486.659832533498</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="13" x14ac:dyDescent="0.15">
       <c r="A4" s="4" t="s">
         <v>19</v>
       </c>
@@ -679,7 +723,7 @@
         <v>49919.895492193667</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="7" t="s">
         <v>38</v>
       </c>
@@ -723,7 +767,7 @@
         <v>79447.705273471176</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="7" t="s">
         <v>39</v>
       </c>
@@ -778,20 +822,20 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:AA17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="30.77734375" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="29.6640625" customWidth="1"/>
-    <col min="3" max="3" width="10.21875" customWidth="1"/>
-    <col min="5" max="5" width="11.44140625" customWidth="1"/>
+    <col min="3" max="3" width="10.1640625" customWidth="1"/>
+    <col min="5" max="5" width="11.5" customWidth="1"/>
     <col min="6" max="6" width="10.6640625" customWidth="1"/>
-    <col min="7" max="7" width="19.109375" customWidth="1"/>
-    <col min="8" max="8" width="19.88671875" customWidth="1"/>
-    <col min="9" max="9" width="21.109375" customWidth="1"/>
-    <col min="10" max="12" width="19.109375" customWidth="1"/>
+    <col min="7" max="7" width="19.1640625" customWidth="1"/>
+    <col min="8" max="8" width="19.83203125" customWidth="1"/>
+    <col min="9" max="9" width="21.1640625" customWidth="1"/>
+    <col min="10" max="12" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="31.2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="34" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -844,7 +888,7 @@
       <c r="Z1" s="3"/>
       <c r="AA1" s="3"/>
     </row>
-    <row r="2" spans="1:27" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" ht="13" x14ac:dyDescent="0.15">
       <c r="A2" s="8" t="s">
         <v>27</v>
       </c>
@@ -886,7 +930,7 @@
       </c>
       <c r="M2" s="11"/>
     </row>
-    <row r="3" spans="1:27" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" ht="13" x14ac:dyDescent="0.15">
       <c r="A3" s="8" t="s">
         <v>30</v>
       </c>
@@ -928,7 +972,7 @@
       </c>
       <c r="M3" s="11"/>
     </row>
-    <row r="4" spans="1:27" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" ht="13" x14ac:dyDescent="0.15">
       <c r="A4" s="8" t="s">
         <v>32</v>
       </c>
@@ -970,7 +1014,7 @@
       </c>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="1:27" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" ht="13" x14ac:dyDescent="0.15">
       <c r="A5" s="8" t="s">
         <v>34</v>
       </c>
@@ -1012,7 +1056,7 @@
       </c>
       <c r="M5" s="11"/>
     </row>
-    <row r="6" spans="1:27" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" ht="13" x14ac:dyDescent="0.15">
       <c r="A6" s="8" t="s">
         <v>36</v>
       </c>
@@ -1054,42 +1098,127 @@
       </c>
       <c r="M6" s="11"/>
     </row>
-    <row r="8" spans="1:27" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="E8" s="8"/>
-    </row>
-    <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-    </row>
-    <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-    </row>
-    <row r="11" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-    </row>
-    <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="13">
+        <v>-113.3917</v>
+      </c>
+      <c r="F7" s="13">
+        <v>53.546100000000003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="13">
+        <v>-80.051699999999997</v>
+      </c>
+      <c r="F8" s="13">
+        <v>42.837499999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" s="13">
+        <v>-82.415999999999997</v>
+      </c>
+      <c r="F9" s="13">
+        <v>42.951900000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="13">
+        <v>-110.47199999999999</v>
+      </c>
+      <c r="F10" s="13">
+        <v>54.612099999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="13">
+        <v>-111.24639999999999</v>
+      </c>
+      <c r="F11" s="13">
+        <v>57.295200000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
     </row>
-    <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
     </row>
-    <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
     </row>
-    <row r="16" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
     </row>
-    <row r="17" spans="6:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="6:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="F17" s="8"/>
     </row>
   </sheetData>
@@ -1103,7 +1232,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>